<commit_message>
Atualizando a develop com a ultima feature postada (consultarContrato/M.I)
</commit_message>
<xml_diff>
--- a/db/OLEO26.xlsx
+++ b/db/OLEO26.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D9E0E2-4AE6-43BD-BA08-477831434E56}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E991608-C53C-4F18-B6C4-A36D3A57C22F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2358,8 +2358,15 @@
     <col min="8" max="8" width="11.44140625" style="3" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" style="2" customWidth="1"/>
     <col min="10" max="10" width="50" style="1" customWidth="1"/>
-    <col min="11" max="16" width="11.44140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.44140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="31.21875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="15.77734375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="53.21875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="28" style="1" customWidth="1"/>
+    <col min="16" max="16" width="67.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="19.21875" customWidth="1"/>
+    <col min="18" max="18" width="19.33203125" customWidth="1"/>
+    <col min="21" max="21" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualizando essa branch com a develop
</commit_message>
<xml_diff>
--- a/db/OLEO26.xlsx
+++ b/db/OLEO26.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D9E0E2-4AE6-43BD-BA08-477831434E56}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E991608-C53C-4F18-B6C4-A36D3A57C22F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2358,8 +2358,15 @@
     <col min="8" max="8" width="11.44140625" style="3" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" style="2" customWidth="1"/>
     <col min="10" max="10" width="50" style="1" customWidth="1"/>
-    <col min="11" max="16" width="11.44140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.44140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="31.21875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="15.77734375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="53.21875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="28" style="1" customWidth="1"/>
+    <col min="16" max="16" width="67.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="19.21875" customWidth="1"/>
+    <col min="18" max="18" width="19.33203125" customWidth="1"/>
+    <col min="21" max="21" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">

</xml_diff>